<commit_message>
All tables for Chapter 3 committed
- Table 3 committed
</commit_message>
<xml_diff>
--- a/output/Chp3_tables/Chp3 - Table2.xlsx
+++ b/output/Chp3_tables/Chp3 - Table2.xlsx
@@ -73,190 +73,190 @@
     <t>Expansion scenario - 60% access to POC VL testing, with DR testing both before treatment initiation and confirm treatment failure</t>
   </si>
   <si>
-    <t>47.2 (22.6 - 115.6)</t>
-  </si>
-  <si>
-    <t>49.8 (24.8 - 119.8)</t>
-  </si>
-  <si>
-    <t>52.7 (26.8 - 124.3)</t>
-  </si>
-  <si>
-    <t>55.2 (28.8 - 129.3)</t>
-  </si>
-  <si>
-    <t>57.9 (29.8 - 142.8)</t>
-  </si>
-  <si>
-    <t>68.2 (36.1 - 169.2)</t>
-  </si>
-  <si>
-    <t>77.8 (42.6 - 188.2)</t>
-  </si>
-  <si>
-    <t>52.4 (27.0 - 122.2)</t>
-  </si>
-  <si>
-    <t>55.9 (29.9 - 127.4)</t>
-  </si>
-  <si>
-    <t>58.7 (32.2 - 130.3)</t>
-  </si>
-  <si>
-    <t>59.5 (31.3 - 142.9)</t>
-  </si>
-  <si>
-    <t>68.6 (37.6 - 162.3)</t>
-  </si>
-  <si>
-    <t>76.4 (43.3 - 179.5)</t>
-  </si>
-  <si>
-    <t>2.6 (0.8 - 5.8)</t>
-  </si>
-  <si>
-    <t>5.5 (1.9 - 11.7)</t>
-  </si>
-  <si>
-    <t>8.1 (3.2 - 17.8)</t>
-  </si>
-  <si>
-    <t>10.7 (5.4 - 33.0)</t>
-  </si>
-  <si>
-    <t>21.0 (10.7 - 61.7)</t>
-  </si>
-  <si>
-    <t>30.6 (15.8 - 88.5)</t>
-  </si>
-  <si>
-    <t>5.2 (1.8 - 11.7)</t>
-  </si>
-  <si>
-    <t>8.7 (3.0 - 19.3)</t>
-  </si>
-  <si>
-    <t>11.5 (4.3 - 25.0)</t>
-  </si>
-  <si>
-    <t>12.3 (6.4 - 34.1)</t>
-  </si>
-  <si>
-    <t>21.4 (11.6 - 61.2)</t>
-  </si>
-  <si>
-    <t>29.2 (15.9 - 81.4)</t>
-  </si>
-  <si>
-    <t>27,959 (15,141 - 47,770)</t>
-  </si>
-  <si>
-    <t>27,956 (15,123 - 47,762)</t>
-  </si>
-  <si>
-    <t>27,953 (15,109 - 47,757)</t>
-  </si>
-  <si>
-    <t>27,952 (15,099 - 47,753)</t>
-  </si>
-  <si>
-    <t>27,949 (15,110 - 47,754)</t>
-  </si>
-  <si>
-    <t>27,940 (15,095 - 47,738)</t>
-  </si>
-  <si>
-    <t>27,931 (15,082 - 47,723)</t>
-  </si>
-  <si>
-    <t>27,938 (15,092 - 47,740)</t>
-  </si>
-  <si>
-    <t>27,925 (15,081 - 47,720)</t>
-  </si>
-  <si>
-    <t>27,916 (15,072 - 47,707)</t>
-  </si>
-  <si>
-    <t>27,933 (15,089 - 47,734)</t>
-  </si>
-  <si>
-    <t>27,918 (15,078 - 47,712)</t>
-  </si>
-  <si>
-    <t>27,903 (15,067 - 47,696)</t>
-  </si>
-  <si>
-    <t>3,445 (1,071 - 23,635)</t>
-  </si>
-  <si>
-    <t>5,818 (1,755 - 39,399)</t>
-  </si>
-  <si>
-    <t>7,555 (2,242 - 51,575)</t>
-  </si>
-  <si>
-    <t>10,176 (1,816 - 42,822)</t>
-  </si>
-  <si>
-    <t>19,527 (3,172 - 82,714)</t>
-  </si>
-  <si>
-    <t>28,296 (4,503 - 119,845)</t>
-  </si>
-  <si>
-    <t>21,211 (3,815 - 80,829)</t>
-  </si>
-  <si>
-    <t>34,147 (5,774 - 130,791)</t>
-  </si>
-  <si>
-    <t>42,998 (6,786 - 165,340)</t>
-  </si>
-  <si>
-    <t>26,059 (4,065 - 96,052)</t>
-  </si>
-  <si>
-    <t>41,772 (6,213 - 157,475)</t>
-  </si>
-  <si>
-    <t>56,782 (7,315 - 197,212)</t>
-  </si>
-  <si>
-    <t>750 (44 - 1,865)</t>
-  </si>
-  <si>
-    <t>949 (64 - 2,261)</t>
-  </si>
-  <si>
-    <t>1,066 (83 - 2,639)</t>
-  </si>
-  <si>
-    <t>1,054 (330 - 3,671)</t>
-  </si>
-  <si>
-    <t>1,078 (357 - 4,015)</t>
-  </si>
-  <si>
-    <t>1,082 (344 - 4,227)</t>
-  </si>
-  <si>
-    <t>244 (21 - 983)</t>
-  </si>
-  <si>
-    <t>255 (22 - 1,095)</t>
-  </si>
-  <si>
-    <t>268 (25 - 1,211)</t>
-  </si>
-  <si>
-    <t>473 (146 - 1,991)</t>
-  </si>
-  <si>
-    <t>513 (155 - 2,372)</t>
-  </si>
-  <si>
-    <t>515 (169 - 2,739)</t>
+    <t>47.7 (23.4 - 106.8)</t>
+  </si>
+  <si>
+    <t>50.2 (25.6 - 109.6)</t>
+  </si>
+  <si>
+    <t>53.3 (27.3 - 112.7)</t>
+  </si>
+  <si>
+    <t>56.2 (30.2 - 115.3)</t>
+  </si>
+  <si>
+    <t>58.7 (31.0 - 123.5)</t>
+  </si>
+  <si>
+    <t>69.1 (38.2 - 143.2)</t>
+  </si>
+  <si>
+    <t>79.9 (45.1 - 167.9)</t>
+  </si>
+  <si>
+    <t>52.9 (27.7 - 112.9)</t>
+  </si>
+  <si>
+    <t>57.2 (31.7 - 116.2)</t>
+  </si>
+  <si>
+    <t>60.6 (34.0 - 118.9)</t>
+  </si>
+  <si>
+    <t>60.8 (32.6 - 123.5)</t>
+  </si>
+  <si>
+    <t>71.2 (39.7 - 144.4)</t>
+  </si>
+  <si>
+    <t>80.4 (45.5 - 163.6)</t>
+  </si>
+  <si>
+    <t>2.5 (1.1 - 5.8)</t>
+  </si>
+  <si>
+    <t>5.6 (2.4 - 11.7)</t>
+  </si>
+  <si>
+    <t>8.4 (3.6 - 17.7)</t>
+  </si>
+  <si>
+    <t>10.9 (5.7 - 24.4)</t>
+  </si>
+  <si>
+    <t>21.4 (11.3 - 47.8)</t>
+  </si>
+  <si>
+    <t>32.1 (16.8 - 69.7)</t>
+  </si>
+  <si>
+    <t>5.2 (2.7 - 10.1)</t>
+  </si>
+  <si>
+    <t>9.5 (4.7 - 16.9)</t>
+  </si>
+  <si>
+    <t>12.9 (6.5 - 23.0)</t>
+  </si>
+  <si>
+    <t>13.0 (7.0 - 27.2)</t>
+  </si>
+  <si>
+    <t>23.4 (12.7 - 48.2)</t>
+  </si>
+  <si>
+    <t>32.6 (17.9 - 67.0)</t>
+  </si>
+  <si>
+    <t>28,664 (17,125 - 46,487)</t>
+  </si>
+  <si>
+    <t>28,658 (17,114 - 46,483)</t>
+  </si>
+  <si>
+    <t>28,654 (17,106 - 46,480)</t>
+  </si>
+  <si>
+    <t>28,651 (17,100 - 46,478)</t>
+  </si>
+  <si>
+    <t>28,652 (17,101 - 46,479)</t>
+  </si>
+  <si>
+    <t>28,640 (17,079 - 46,471)</t>
+  </si>
+  <si>
+    <t>28,630 (17,059 - 46,465)</t>
+  </si>
+  <si>
+    <t>28,635 (17,046 - 46,469)</t>
+  </si>
+  <si>
+    <t>28,618 (17,005 - 46,460)</t>
+  </si>
+  <si>
+    <t>28,614 (16,980 - 46,454)</t>
+  </si>
+  <si>
+    <t>28,631 (17,038 - 46,467)</t>
+  </si>
+  <si>
+    <t>28,617 (16,994 - 46,456)</t>
+  </si>
+  <si>
+    <t>28,612 (16,968 - 46,449)</t>
+  </si>
+  <si>
+    <t>6,311 (2,157 - 25,271)</t>
+  </si>
+  <si>
+    <t>10,642 (3,695 - 42,499)</t>
+  </si>
+  <si>
+    <t>13,806 (4,867 - 56,342)</t>
+  </si>
+  <si>
+    <t>12,789 (2,934 - 38,732)</t>
+  </si>
+  <si>
+    <t>24,194 (5,221 - 71,841)</t>
+  </si>
+  <si>
+    <t>34,696 (7,230 - 100,828)</t>
+  </si>
+  <si>
+    <t>29,000 (6,061 - 69,013)</t>
+  </si>
+  <si>
+    <t>45,987 (9,690 - 113,279)</t>
+  </si>
+  <si>
+    <t>50,697 (12,084 - 142,605)</t>
+  </si>
+  <si>
+    <t>33,656 (6,374 - 81,254)</t>
+  </si>
+  <si>
+    <t>47,373 (10,165 - 130,347)</t>
+  </si>
+  <si>
+    <t>52,269 (12,791 - 162,589)</t>
+  </si>
+  <si>
+    <t>398 (80 - 1,446)</t>
+  </si>
+  <si>
+    <t>524 (101 - 1,699)</t>
+  </si>
+  <si>
+    <t>612 (123 - 1,963)</t>
+  </si>
+  <si>
+    <t>855 (351 - 3,263)</t>
+  </si>
+  <si>
+    <t>884 (377 - 3,587)</t>
+  </si>
+  <si>
+    <t>926 (397 - 3,851)</t>
+  </si>
+  <si>
+    <t>179 (73 - 818)</t>
+  </si>
+  <si>
+    <t>206 (77 - 921)</t>
+  </si>
+  <si>
+    <t>254 (83 - 1,047)</t>
+  </si>
+  <si>
+    <t>387 (197 - 1,695)</t>
+  </si>
+  <si>
+    <t>495 (214 - 1,969)</t>
+  </si>
+  <si>
+    <t>624 (237 - 2,209)</t>
   </si>
 </sst>
 </file>

</xml_diff>